<commit_message>
Add regional spillover in local learning
Add a new variable for regional spillover effects in learning calculation. This is so that policies in cities can influence national cost declines.

Tweaking gamma values for freight.

Also adjusting stringency effect of HDT BEV sales mandate to 2/3 of max mandate (up from 1/2).
</commit_message>
<xml_diff>
--- a/Inputs/_MasterFiles/FTT_variables.xlsx
+++ b/Inputs/_MasterFiles/FTT_variables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofexeteruk-my.sharepoint.com/personal/f_j_m_m_nijsse_exeter_ac_uk/Documents/Documents/GitHub/FTT_StandAlone/Inputs/_MasterFiles/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\FTT_StandAlone\Inputs\_MasterFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{96C6DCC7-F135-4F9F-BBD1-97530C10B60C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5C4C47A-7846-4D5B-9B0B-09EFC23E3A8E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6E6CE53-B410-4DDA-B35B-F2962674C9CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FTT-P" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="748" uniqueCount="276">
   <si>
     <t>Variable name</t>
   </si>
@@ -858,6 +858,18 @@
   </si>
   <si>
     <t>FTT-Tr relative registration tax or subsidy</t>
+  </si>
+  <si>
+    <t>FTT-Fr City mapping</t>
+  </si>
+  <si>
+    <t>city mapping</t>
+  </si>
+  <si>
+    <t>region spillover</t>
+  </si>
+  <si>
+    <t>FTT-Fr Regional spillover matrix</t>
   </si>
 </sst>
 </file>
@@ -3662,12 +3674,12 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85BB7FF7-82D6-482E-815B-F3751454FF7D}">
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="37.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="29" customWidth="1"/>
@@ -4297,14 +4309,73 @@
         <v>260</v>
       </c>
     </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>273</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19">
+        <v>35430000</v>
+      </c>
+      <c r="D19" t="s">
+        <v>272</v>
+      </c>
+      <c r="E19" t="s">
+        <v>54</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="J19" t="s">
+        <v>24</v>
+      </c>
+      <c r="K19" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>274</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20">
+        <v>35440000</v>
+      </c>
+      <c r="D20" t="s">
+        <v>275</v>
+      </c>
+      <c r="E20" t="s">
+        <v>54</v>
+      </c>
+      <c r="F20" t="s">
+        <v>54</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20" t="s">
+        <v>260</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA629D80-511C-42AD-ACB3-22237E3BD282}">
-  <dimension ref="A1:B67"/>
+  <dimension ref="A1:B68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -4840,6 +4911,14 @@
         <v>266</v>
       </c>
       <c r="B67" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>273</v>
+      </c>
+      <c r="B68" t="s">
         <v>248</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add script to generate values for sensitivity analysis
Plus update ftt_variables to create bztc csvs for every scenario (need to find better solution as this is not needed for majority of scenarios)
</commit_message>
<xml_diff>
--- a/Inputs/_MasterFiles/FTT_variables.xlsx
+++ b/Inputs/_MasterFiles/FTT_variables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\FTT_StandAlone\Inputs\_MasterFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6E6CE53-B410-4DDA-B35B-F2962674C9CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3DF6274-83FA-405B-AF6B-8FAA23447639}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4242,7 +4242,7 @@
         <v>257</v>
       </c>
       <c r="K16" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add spreadsheet for fuel price adjustment
For FTT-Heat. Fuel prices in BE, DE, UK adjusted to achieve spark price of no more than 2.

Updated FTT_variables to extract heat cost matrix on all scenarios.
</commit_message>
<xml_diff>
--- a/Inputs/_MasterFiles/FTT_variables.xlsx
+++ b/Inputs/_MasterFiles/FTT_variables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofexeteruk-my.sharepoint.com/personal/f_j_m_m_nijsse_exeter_ac_uk/Documents/Documents/GitHub/FTT_StandAlone/Inputs/_MasterFiles/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\FTT_StandAlone\Inputs\_MasterFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{96C6DCC7-F135-4F9F-BBD1-97530C10B60C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5C4C47A-7846-4D5B-9B0B-09EFC23E3A8E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3FF3758-B89F-41AC-AD73-A8A9FB5F181D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FTT-P" sheetId="1" r:id="rId1"/>
@@ -1189,16 +1189,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="35" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" customWidth="1"/>
+    <col min="6" max="6" width="12.81640625" customWidth="1"/>
+    <col min="7" max="7" width="14.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1227,7 +1227,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1256,7 +1256,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>58</v>
       </c>
@@ -1285,7 +1285,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>62</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>63</v>
       </c>
@@ -1343,7 +1343,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>73</v>
       </c>
@@ -1372,7 +1372,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>83</v>
       </c>
@@ -1401,7 +1401,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>55</v>
       </c>
@@ -1430,7 +1430,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>78</v>
       </c>
@@ -1459,7 +1459,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>69</v>
       </c>
@@ -1488,7 +1488,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>71</v>
       </c>
@@ -1517,7 +1517,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>67</v>
       </c>
@@ -1546,7 +1546,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>80</v>
       </c>
@@ -1575,7 +1575,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>87</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>89</v>
       </c>
@@ -1633,7 +1633,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>79</v>
       </c>
@@ -1662,7 +1662,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>81</v>
       </c>
@@ -1691,7 +1691,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>75</v>
       </c>
@@ -1734,14 +1734,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E04294AC-DBC1-4E51-84ED-2EC5066B9024}">
   <dimension ref="A1:I23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="46.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="46.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1770,7 +1770,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1799,7 +1799,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -1828,7 +1828,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1857,7 +1857,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1886,7 +1886,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1915,7 +1915,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -1944,7 +1944,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>270</v>
       </c>
@@ -1973,7 +1973,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -2002,7 +2002,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -2031,7 +2031,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -2060,7 +2060,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -2089,7 +2089,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -2118,7 +2118,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>31</v>
       </c>
@@ -2147,7 +2147,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -2176,7 +2176,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>33</v>
       </c>
@@ -2205,7 +2205,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -2234,7 +2234,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>35</v>
       </c>
@@ -2263,7 +2263,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -2292,7 +2292,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -2321,7 +2321,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>36</v>
       </c>
@@ -2350,7 +2350,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>16</v>
       </c>
@@ -2379,7 +2379,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>52</v>
       </c>
@@ -2416,13 +2416,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{893746F0-70F0-4C21-8E46-9B5DBA6E54BB}">
   <dimension ref="A1:I17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.42578125" customWidth="1"/>
+    <col min="2" max="2" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>95</v>
       </c>
@@ -2480,7 +2480,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>98</v>
       </c>
@@ -2509,7 +2509,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>99</v>
       </c>
@@ -2538,7 +2538,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>100</v>
       </c>
@@ -2567,7 +2567,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>101</v>
       </c>
@@ -2596,7 +2596,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>102</v>
       </c>
@@ -2625,7 +2625,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>103</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>104</v>
       </c>
@@ -2683,7 +2683,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>105</v>
       </c>
@@ -2712,7 +2712,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>106</v>
       </c>
@@ -2741,7 +2741,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>107</v>
       </c>
@@ -2770,7 +2770,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>108</v>
       </c>
@@ -2799,7 +2799,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>109</v>
       </c>
@@ -2828,7 +2828,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>110</v>
       </c>
@@ -2857,7 +2857,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>111</v>
       </c>
@@ -2886,7 +2886,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>112</v>
       </c>
@@ -2912,7 +2912,7 @@
         <v>257</v>
       </c>
       <c r="I17" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>
@@ -2923,14 +2923,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F76D307B-9060-4C33-AF9D-2A846C2CA587}">
   <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="50.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="50.54296875" customWidth="1"/>
+    <col min="5" max="5" width="9.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2959,7 +2959,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>130</v>
       </c>
@@ -2988,7 +2988,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>154</v>
       </c>
@@ -3017,7 +3017,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>131</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>132</v>
       </c>
@@ -3075,7 +3075,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>133</v>
       </c>
@@ -3104,7 +3104,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>134</v>
       </c>
@@ -3133,7 +3133,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>135</v>
       </c>
@@ -3162,7 +3162,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>136</v>
       </c>
@@ -3191,7 +3191,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>137</v>
       </c>
@@ -3220,7 +3220,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>138</v>
       </c>
@@ -3249,7 +3249,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>139</v>
       </c>
@@ -3278,7 +3278,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>140</v>
       </c>
@@ -3307,7 +3307,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>141</v>
       </c>
@@ -3336,7 +3336,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>142</v>
       </c>
@@ -3365,7 +3365,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>143</v>
       </c>
@@ -3394,7 +3394,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>144</v>
       </c>
@@ -3423,7 +3423,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>145</v>
       </c>
@@ -3452,7 +3452,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>146</v>
       </c>
@@ -3481,7 +3481,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>147</v>
       </c>
@@ -3510,7 +3510,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>148</v>
       </c>
@@ -3539,7 +3539,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>149</v>
       </c>
@@ -3568,7 +3568,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>150</v>
       </c>
@@ -3597,7 +3597,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>151</v>
       </c>
@@ -3626,7 +3626,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>152</v>
       </c>
@@ -3663,17 +3663,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85BB7FF7-82D6-482E-815B-F3751454FF7D}">
   <dimension ref="A1:K18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="37.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.54296875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3708,7 +3708,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>188</v>
       </c>
@@ -3743,7 +3743,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>213</v>
       </c>
@@ -3778,7 +3778,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>265</v>
       </c>
@@ -3813,7 +3813,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>212</v>
       </c>
@@ -3848,7 +3848,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>214</v>
       </c>
@@ -3883,7 +3883,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>215</v>
       </c>
@@ -3918,7 +3918,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>216</v>
       </c>
@@ -3953,7 +3953,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>217</v>
       </c>
@@ -3988,7 +3988,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>218</v>
       </c>
@@ -4023,7 +4023,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>226</v>
       </c>
@@ -4058,7 +4058,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>227</v>
       </c>
@@ -4093,7 +4093,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>231</v>
       </c>
@@ -4128,7 +4128,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>240</v>
       </c>
@@ -4163,7 +4163,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>236</v>
       </c>
@@ -4198,7 +4198,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>269</v>
       </c>
@@ -4233,7 +4233,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>249</v>
       </c>
@@ -4268,7 +4268,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>266</v>
       </c>
@@ -4305,9 +4305,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA629D80-511C-42AD-ACB3-22237E3BD282}">
   <dimension ref="A1:B67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4315,7 +4315,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -4323,7 +4323,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>36</v>
       </c>
@@ -4331,7 +4331,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -4339,7 +4339,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -4347,7 +4347,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -4355,7 +4355,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>52</v>
       </c>
@@ -4363,7 +4363,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>26</v>
       </c>
@@ -4371,7 +4371,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -4379,7 +4379,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>270</v>
       </c>
@@ -4387,7 +4387,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -4395,7 +4395,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -4403,7 +4403,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -4411,7 +4411,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -4419,7 +4419,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>58</v>
       </c>
@@ -4427,7 +4427,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>62</v>
       </c>
@@ -4435,7 +4435,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>63</v>
       </c>
@@ -4443,7 +4443,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>73</v>
       </c>
@@ -4451,7 +4451,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>78</v>
       </c>
@@ -4459,7 +4459,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>69</v>
       </c>
@@ -4467,7 +4467,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>71</v>
       </c>
@@ -4475,7 +4475,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>67</v>
       </c>
@@ -4483,7 +4483,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>66</v>
       </c>
@@ -4491,7 +4491,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>75</v>
       </c>
@@ -4499,7 +4499,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>102</v>
       </c>
@@ -4507,7 +4507,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>103</v>
       </c>
@@ -4515,7 +4515,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>104</v>
       </c>
@@ -4523,7 +4523,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>105</v>
       </c>
@@ -4531,7 +4531,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>106</v>
       </c>
@@ -4539,7 +4539,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>107</v>
       </c>
@@ -4547,7 +4547,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>108</v>
       </c>
@@ -4555,7 +4555,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>109</v>
       </c>
@@ -4563,7 +4563,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>110</v>
       </c>
@@ -4571,7 +4571,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>111</v>
       </c>
@@ -4579,7 +4579,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>129</v>
       </c>
@@ -4587,7 +4587,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>130</v>
       </c>
@@ -4595,7 +4595,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>154</v>
       </c>
@@ -4603,7 +4603,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>131</v>
       </c>
@@ -4611,7 +4611,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>146</v>
       </c>
@@ -4619,7 +4619,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>147</v>
       </c>
@@ -4627,7 +4627,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>148</v>
       </c>
@@ -4635,7 +4635,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>149</v>
       </c>
@@ -4643,7 +4643,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>150</v>
       </c>
@@ -4651,7 +4651,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>151</v>
       </c>
@@ -4659,7 +4659,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>152</v>
       </c>
@@ -4667,7 +4667,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>185</v>
       </c>
@@ -4675,7 +4675,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>188</v>
       </c>
@@ -4683,7 +4683,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>213</v>
       </c>
@@ -4691,7 +4691,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>192</v>
       </c>
@@ -4699,7 +4699,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>265</v>
       </c>
@@ -4707,7 +4707,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>212</v>
       </c>
@@ -4715,7 +4715,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>214</v>
       </c>
@@ -4723,7 +4723,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>215</v>
       </c>
@@ -4731,7 +4731,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>216</v>
       </c>
@@ -4739,7 +4739,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>217</v>
       </c>
@@ -4747,7 +4747,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>218</v>
       </c>
@@ -4755,7 +4755,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>230</v>
       </c>
@@ -4763,7 +4763,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>231</v>
       </c>
@@ -4771,7 +4771,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>235</v>
       </c>
@@ -4779,7 +4779,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>240</v>
       </c>
@@ -4787,7 +4787,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>31</v>
       </c>
@@ -4795,7 +4795,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>254</v>
       </c>
@@ -4803,7 +4803,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>258</v>
       </c>
@@ -4811,7 +4811,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>263</v>
       </c>
@@ -4819,7 +4819,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>249</v>
       </c>
@@ -4827,7 +4827,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>101</v>
       </c>
@@ -4835,7 +4835,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>266</v>
       </c>

</xml_diff>

<commit_message>
Revert "Add spreadsheet for fuel price adjustment"
This reverts commit 6286403ca835f488ae06cf0f340e77506b5e6519.
</commit_message>
<xml_diff>
--- a/Inputs/_MasterFiles/FTT_variables.xlsx
+++ b/Inputs/_MasterFiles/FTT_variables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\FTT_StandAlone\Inputs\_MasterFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofexeteruk-my.sharepoint.com/personal/f_j_m_m_nijsse_exeter_ac_uk/Documents/Documents/GitHub/FTT_StandAlone/Inputs/_MasterFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3FF3758-B89F-41AC-AD73-A8A9FB5F181D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{96C6DCC7-F135-4F9F-BBD1-97530C10B60C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5C4C47A-7846-4D5B-9B0B-09EFC23E3A8E}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FTT-P" sheetId="1" r:id="rId1"/>
@@ -1189,16 +1189,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="35" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="12.81640625" customWidth="1"/>
-    <col min="7" max="7" width="14.453125" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1227,7 +1227,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1256,7 +1256,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>58</v>
       </c>
@@ -1285,7 +1285,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>62</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>63</v>
       </c>
@@ -1343,7 +1343,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>73</v>
       </c>
@@ -1372,7 +1372,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>83</v>
       </c>
@@ -1401,7 +1401,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>55</v>
       </c>
@@ -1430,7 +1430,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>78</v>
       </c>
@@ -1459,7 +1459,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>69</v>
       </c>
@@ -1488,7 +1488,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>71</v>
       </c>
@@ -1517,7 +1517,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>67</v>
       </c>
@@ -1546,7 +1546,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>80</v>
       </c>
@@ -1575,7 +1575,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>87</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>89</v>
       </c>
@@ -1633,7 +1633,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>79</v>
       </c>
@@ -1662,7 +1662,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>81</v>
       </c>
@@ -1691,7 +1691,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>75</v>
       </c>
@@ -1734,14 +1734,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E04294AC-DBC1-4E51-84ED-2EC5066B9024}">
   <dimension ref="A1:I23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="46.7265625" customWidth="1"/>
+    <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="46.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1770,7 +1770,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1799,7 +1799,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -1828,7 +1828,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1857,7 +1857,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1886,7 +1886,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1915,7 +1915,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -1944,7 +1944,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>270</v>
       </c>
@@ -1973,7 +1973,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -2002,7 +2002,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -2031,7 +2031,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -2060,7 +2060,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -2089,7 +2089,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -2118,7 +2118,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>31</v>
       </c>
@@ -2147,7 +2147,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -2176,7 +2176,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>33</v>
       </c>
@@ -2205,7 +2205,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -2234,7 +2234,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>35</v>
       </c>
@@ -2263,7 +2263,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -2292,7 +2292,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -2321,7 +2321,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>36</v>
       </c>
@@ -2350,7 +2350,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>16</v>
       </c>
@@ -2379,7 +2379,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>52</v>
       </c>
@@ -2416,13 +2416,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{893746F0-70F0-4C21-8E46-9B5DBA6E54BB}">
   <dimension ref="A1:I17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.453125" customWidth="1"/>
+    <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>95</v>
       </c>
@@ -2480,7 +2480,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>98</v>
       </c>
@@ -2509,7 +2509,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>99</v>
       </c>
@@ -2538,7 +2538,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>100</v>
       </c>
@@ -2567,7 +2567,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>101</v>
       </c>
@@ -2596,7 +2596,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>102</v>
       </c>
@@ -2625,7 +2625,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>103</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>104</v>
       </c>
@@ -2683,7 +2683,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>105</v>
       </c>
@@ -2712,7 +2712,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>106</v>
       </c>
@@ -2741,7 +2741,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>107</v>
       </c>
@@ -2770,7 +2770,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>108</v>
       </c>
@@ -2799,7 +2799,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>109</v>
       </c>
@@ -2828,7 +2828,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>110</v>
       </c>
@@ -2857,7 +2857,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>111</v>
       </c>
@@ -2886,7 +2886,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>112</v>
       </c>
@@ -2912,7 +2912,7 @@
         <v>257</v>
       </c>
       <c r="I17" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>
@@ -2923,14 +2923,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F76D307B-9060-4C33-AF9D-2A846C2CA587}">
   <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="50.54296875" customWidth="1"/>
-    <col min="5" max="5" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="50.5703125" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2959,7 +2959,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>130</v>
       </c>
@@ -2988,7 +2988,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>154</v>
       </c>
@@ -3017,7 +3017,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>131</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>132</v>
       </c>
@@ -3075,7 +3075,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>133</v>
       </c>
@@ -3104,7 +3104,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>134</v>
       </c>
@@ -3133,7 +3133,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>135</v>
       </c>
@@ -3162,7 +3162,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>136</v>
       </c>
@@ -3191,7 +3191,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>137</v>
       </c>
@@ -3220,7 +3220,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>138</v>
       </c>
@@ -3249,7 +3249,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>139</v>
       </c>
@@ -3278,7 +3278,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>140</v>
       </c>
@@ -3307,7 +3307,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>141</v>
       </c>
@@ -3336,7 +3336,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>142</v>
       </c>
@@ -3365,7 +3365,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>143</v>
       </c>
@@ -3394,7 +3394,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>144</v>
       </c>
@@ -3423,7 +3423,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>145</v>
       </c>
@@ -3452,7 +3452,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>146</v>
       </c>
@@ -3481,7 +3481,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>147</v>
       </c>
@@ -3510,7 +3510,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>148</v>
       </c>
@@ -3539,7 +3539,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>149</v>
       </c>
@@ -3568,7 +3568,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>150</v>
       </c>
@@ -3597,7 +3597,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>151</v>
       </c>
@@ -3626,7 +3626,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>152</v>
       </c>
@@ -3663,17 +3663,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85BB7FF7-82D6-482E-815B-F3751454FF7D}">
   <dimension ref="A1:K18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="37.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3708,7 +3708,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>188</v>
       </c>
@@ -3743,7 +3743,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>213</v>
       </c>
@@ -3778,7 +3778,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>265</v>
       </c>
@@ -3813,7 +3813,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>212</v>
       </c>
@@ -3848,7 +3848,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>214</v>
       </c>
@@ -3883,7 +3883,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>215</v>
       </c>
@@ -3918,7 +3918,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>216</v>
       </c>
@@ -3953,7 +3953,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>217</v>
       </c>
@@ -3988,7 +3988,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>218</v>
       </c>
@@ -4023,7 +4023,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>226</v>
       </c>
@@ -4058,7 +4058,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>227</v>
       </c>
@@ -4093,7 +4093,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>231</v>
       </c>
@@ -4128,7 +4128,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>240</v>
       </c>
@@ -4163,7 +4163,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>236</v>
       </c>
@@ -4198,7 +4198,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>269</v>
       </c>
@@ -4233,7 +4233,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>249</v>
       </c>
@@ -4268,7 +4268,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>266</v>
       </c>
@@ -4305,9 +4305,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA629D80-511C-42AD-ACB3-22237E3BD282}">
   <dimension ref="A1:B67"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4315,7 +4315,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -4323,7 +4323,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>36</v>
       </c>
@@ -4331,7 +4331,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -4339,7 +4339,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -4347,7 +4347,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -4355,7 +4355,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>52</v>
       </c>
@@ -4363,7 +4363,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>26</v>
       </c>
@@ -4371,7 +4371,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -4379,7 +4379,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>270</v>
       </c>
@@ -4387,7 +4387,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -4395,7 +4395,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -4403,7 +4403,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -4411,7 +4411,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -4419,7 +4419,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>58</v>
       </c>
@@ -4427,7 +4427,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>62</v>
       </c>
@@ -4435,7 +4435,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>63</v>
       </c>
@@ -4443,7 +4443,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>73</v>
       </c>
@@ -4451,7 +4451,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>78</v>
       </c>
@@ -4459,7 +4459,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>69</v>
       </c>
@@ -4467,7 +4467,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>71</v>
       </c>
@@ -4475,7 +4475,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>67</v>
       </c>
@@ -4483,7 +4483,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>66</v>
       </c>
@@ -4491,7 +4491,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>75</v>
       </c>
@@ -4499,7 +4499,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>102</v>
       </c>
@@ -4507,7 +4507,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>103</v>
       </c>
@@ -4515,7 +4515,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>104</v>
       </c>
@@ -4523,7 +4523,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>105</v>
       </c>
@@ -4531,7 +4531,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>106</v>
       </c>
@@ -4539,7 +4539,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>107</v>
       </c>
@@ -4547,7 +4547,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>108</v>
       </c>
@@ -4555,7 +4555,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>109</v>
       </c>
@@ -4563,7 +4563,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>110</v>
       </c>
@@ -4571,7 +4571,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>111</v>
       </c>
@@ -4579,7 +4579,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>129</v>
       </c>
@@ -4587,7 +4587,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>130</v>
       </c>
@@ -4595,7 +4595,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>154</v>
       </c>
@@ -4603,7 +4603,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>131</v>
       </c>
@@ -4611,7 +4611,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>146</v>
       </c>
@@ -4619,7 +4619,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>147</v>
       </c>
@@ -4627,7 +4627,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>148</v>
       </c>
@@ -4635,7 +4635,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>149</v>
       </c>
@@ -4643,7 +4643,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>150</v>
       </c>
@@ -4651,7 +4651,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>151</v>
       </c>
@@ -4659,7 +4659,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>152</v>
       </c>
@@ -4667,7 +4667,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>185</v>
       </c>
@@ -4675,7 +4675,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>188</v>
       </c>
@@ -4683,7 +4683,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>213</v>
       </c>
@@ -4691,7 +4691,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>192</v>
       </c>
@@ -4699,7 +4699,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>265</v>
       </c>
@@ -4707,7 +4707,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>212</v>
       </c>
@@ -4715,7 +4715,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>214</v>
       </c>
@@ -4723,7 +4723,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>215</v>
       </c>
@@ -4731,7 +4731,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>216</v>
       </c>
@@ -4739,7 +4739,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>217</v>
       </c>
@@ -4747,7 +4747,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>218</v>
       </c>
@@ -4755,7 +4755,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>230</v>
       </c>
@@ -4763,7 +4763,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>231</v>
       </c>
@@ -4771,7 +4771,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>235</v>
       </c>
@@ -4779,7 +4779,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>240</v>
       </c>
@@ -4787,7 +4787,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>31</v>
       </c>
@@ -4795,7 +4795,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>254</v>
       </c>
@@ -4803,7 +4803,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>258</v>
       </c>
@@ -4811,7 +4811,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>263</v>
       </c>
@@ -4819,7 +4819,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>249</v>
       </c>
@@ -4827,7 +4827,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>101</v>
       </c>
@@ -4835,7 +4835,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>266</v>
       </c>

</xml_diff>

<commit_message>
Adjusting model structure to add FTT-GMP
ftt_gmp_main solve function runs successfully when called.
</commit_message>
<xml_diff>
--- a/Inputs/_MasterFiles/FTT_variables.xlsx
+++ b/Inputs/_MasterFiles/FTT_variables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofexeteruk-my.sharepoint.com/personal/f_j_m_m_nijsse_exeter_ac_uk/Documents/Documents/GitHub/FTT_StandAlone/Inputs/_MasterFiles/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\FTT_StandAlone_GMP\Inputs\_MasterFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{96C6DCC7-F135-4F9F-BBD1-97530C10B60C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5C4C47A-7846-4D5B-9B0B-09EFC23E3A8E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8E2C91B-3A63-4CFF-9FB4-B7B702B1FFCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FTT-P" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,8 @@
     <sheet name="FTT-H" sheetId="3" r:id="rId3"/>
     <sheet name="FTT-S" sheetId="4" r:id="rId4"/>
     <sheet name="FTT-Fr" sheetId="7" r:id="rId5"/>
-    <sheet name="Time_Horizons" sheetId="6" r:id="rId6"/>
+    <sheet name="FTT-GMP" sheetId="8" r:id="rId6"/>
+    <sheet name="Time_Horizons" sheetId="6" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FTT-P'!$A$1:$G$18</definedName>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="272">
   <si>
     <t>Variable name</t>
   </si>
@@ -4303,6 +4304,59 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A52E5EA-E759-42D2-80A5-71599DAF4092}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>153</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" t="s">
+        <v>186</v>
+      </c>
+      <c r="I1" t="s">
+        <v>187</v>
+      </c>
+      <c r="J1" t="s">
+        <v>256</v>
+      </c>
+      <c r="K1" t="s">
+        <v>259</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA629D80-511C-42AD-ACB3-22237E3BD282}">
   <dimension ref="A1:B67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>